<commit_message>
Templates: new files from a letter, offer, invoice and more
"Neu → Aus Vorlage …" offers built-in templates written as Office XML in
@schreibzeug/ooxml (templates.ts): a letter after DIN 5008, an offer, an
invoice with what § 14 UStG asks of one, a calculation with formulas and
euro formats, a project plan and a presentation. Every document,
spreadsheet and presentation in a folder "Vorlagen" at the top of the
user's files is offered as an own template, on a server as on the
computer.

The new file is the template's bytes uploaded under the name given, so the
API needs nothing new and an own template stays unchanged. xlsx() takes a
few cell styles (bold, euro, date, percent) for the spreadsheets;
preise.xlsx is written again with the new styles part.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019EQFRvL3TVESMctRXTvjbh
</commit_message>
<xml_diff>
--- a/test-files/preise.xlsx
+++ b/test-files/preise.xlsx
@@ -10,8 +10,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="165" formatCode="dd.mm.yyyy"/>
+  </numFmts>
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +47,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>